<commit_message>
integrar IAM y ajustes PCA en indices y homogenizacion
</commit_message>
<xml_diff>
--- a/01_Data/01_Derived/label.xlsx
+++ b/01_Data/01_Derived/label.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B216"/>
+  <dimension ref="A1:B217"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2939,6 +2939,18 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>tasa_iam</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Tasa de mortalidad por infarto agudo de miocardio por cada cien mil habitantes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>